<commit_message>
legacy imaging v3 pipeline: strict injection crosswalks + treatment typing
</commit_message>
<xml_diff>
--- a/seed_kits/legacy_wrangling_v2/raw/Unique_injected_plasmid__preview_dqm.xlsx
+++ b/seed_kits/legacy_wrangling_v2/raw/Unique_injected_plasmid__preview_dqm.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -764,6 +764,78 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>MGCO-49_peroxisome-A2UCOE-ef1aextra-mStayGold-SKL</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>MGCO-49</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>MGCO-28(ef1a-extended-2Xcox8A-linker-mStayGold-SV40-attb-tol2)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>MGCO-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MGCO-01(ef1a-2Xcox8A-linker-mStayGold-SV40-attb-tol2)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MGCO-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MGCO-52-peroxisome-A2UCOE-attb_entire+pDQM147-ABCDpmp70-mStayGold</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MGCO-52, pDQM147</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MGCO54(nuclearenvelope-A2UCOE-attb_entire+pDQM147-LEMD2-mStayGold)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MGCO-54, pDQM147</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>MGCO50(microtubule-A2UCOE-attb_entire+pDQM147-EB3-mStayGold)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MGCO-50, pDQM147</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>